<commit_message>
refactoring eda + stats
</commit_message>
<xml_diff>
--- a/resultados_estatisticos.xlsx
+++ b/resultados_estatisticos.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qui-quadrado e Cramer V" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi2 e Cramer V" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mann-Whitney Salarial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tendência Temporal" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +475,11 @@
           <t>% células (exp≥5)</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Pressuposto OK</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -484,13 +488,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15557</v>
+        <v>12422</v>
       </c>
       <c r="C2" t="n">
-        <v>104.49</v>
+        <v>47.763</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -501,7 +505,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.082</v>
+        <v>0.0607</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -511,6 +515,11 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -538,7 +547,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.1092</v>
+        <v>0.1059</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -548,6 +557,11 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -575,7 +589,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0699</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -585,6 +599,11 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -612,7 +631,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.106</v>
+        <v>0.1037</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -622,6 +641,11 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -649,7 +673,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.0624</v>
+        <v>0.0608</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -659,6 +683,11 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -686,7 +715,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.08260000000000001</v>
+        <v>0.0794</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -696,6 +725,11 @@
       <c r="I7" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -723,7 +757,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.1786</v>
+        <v>0.1773</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -733,6 +767,11 @@
       <c r="I8" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -760,7 +799,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.0318</v>
+        <v>0.0278</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -770,6 +809,11 @@
       <c r="I9" t="inlineStr">
         <is>
           <t>100%</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -784,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,57 +839,52 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>N Masculino</t>
+          <t>N Masc</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>N Feminino</t>
+          <t>N Fem</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Mediana Masc (rank)</t>
+          <t>Mediana Masc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Mediana Fem (rank)</t>
+          <t>Mediana Fem</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Faixa modal Masc</t>
+          <t>U</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Faixa modal Fem</t>
+          <t>p-valor</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>Significativo</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>p-valor</t>
+          <t>r (rank-biserial)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Significativo</t>
+          <t>Direção</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>r (effect size)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Magnitude r</t>
+          <t>Magnitude</t>
         </is>
       </c>
     </row>
@@ -861,48 +900,45 @@
       <c r="C2" t="n">
         <v>3538</v>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>23712840</v>
       </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.1264</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Masc &gt; Fem</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Grande</t>
+          <t>Pequeno</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Brasil — 2021</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -911,46 +947,45 @@
       <c r="C3" t="n">
         <v>430</v>
       </c>
-      <c r="D3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>454266</v>
       </c>
+      <c r="G3" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I3" t="n">
-        <v>6.499999999999999e-05</v>
+        <v>0.1167</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>0.0794</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Negligenciável</t>
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Pequeno</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Brasil — 2022</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -959,46 +994,45 @@
       <c r="C4" t="n">
         <v>876</v>
       </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>1349824</v>
       </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>0.1211</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.0906</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Negligenciável</t>
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Pequeno</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Brasil — 2023</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1007,46 +1041,45 @@
       <c r="C5" t="n">
         <v>1099</v>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>2236891</v>
       </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.1317</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.09760000000000001</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Negligenciável</t>
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Pequeno</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Brasil — 2024</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1055,37 +1088,36 @@
       <c r="C6" t="n">
         <v>1133</v>
       </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="F6" t="n">
         <v>2376175</v>
       </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>0.1454</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1081</v>
-      </c>
-      <c r="L6" t="inlineStr">
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Pequeno</t>
         </is>
@@ -1103,37 +1135,36 @@
       <c r="C7" t="n">
         <v>177</v>
       </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>73175</v>
       </c>
+      <c r="G7" t="n">
+        <v>0.115124</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="I7" t="n">
-        <v>0.057562</v>
+        <v>0.0752</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>0.0512</v>
-      </c>
-      <c r="L7" t="inlineStr">
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>Negligenciável</t>
         </is>
@@ -1151,37 +1182,36 @@
       <c r="C8" t="n">
         <v>341</v>
       </c>
-      <c r="D8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>R$4k-6k</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="F8" t="n">
         <v>242069</v>
       </c>
+      <c r="G8" t="n">
+        <v>4e-06</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I8" t="n">
-        <v>2e-06</v>
+        <v>0.1609</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>0.1162</v>
-      </c>
-      <c r="L8" t="inlineStr">
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>Pequeno</t>
         </is>
@@ -1199,37 +1229,36 @@
       <c r="C9" t="n">
         <v>33</v>
       </c>
-      <c r="D9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>R$4k-6k</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="F9" t="n">
         <v>3425</v>
       </c>
+      <c r="G9" t="n">
+        <v>0.05758</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="I9" t="n">
-        <v>0.02879</v>
+        <v>0.2068</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>0.1326</v>
-      </c>
-      <c r="L9" t="inlineStr">
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>Pequeno</t>
         </is>
@@ -1247,41 +1276,38 @@
       <c r="C10" t="n">
         <v>2283</v>
       </c>
-      <c r="D10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="F10" t="n">
         <v>9290493</v>
       </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>0.1169</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Masc &gt; Fem</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Grande</t>
+          <t>Pequeno</t>
         </is>
       </c>
     </row>
@@ -1297,276 +1323,38 @@
       <c r="C11" t="n">
         <v>629</v>
       </c>
-      <c r="D11" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>R$8k-12k</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>R$8k-12k</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>R$6k-8k</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>800021</v>
       </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>0.1631</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>0.1191</v>
-      </c>
-      <c r="L11" t="inlineStr">
+          <t>Masc &gt; Fem</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>Pequeno</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>β (log-odds/ano)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IC 95% OR</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>p-valor</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Significativo</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Tendência</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Brasil — Geral</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.0585</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1.0603</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[1.025, 1.097]</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0.000711</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Crescente</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Região: Centro-Oeste</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.1135</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1.1202</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[0.971, 1.292]</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0.119501</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Estável</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Região: Nordeste</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.0407</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1.0415</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[0.940, 1.155]</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.439353</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Estável</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Região: Norte</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.0507</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.9505</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[0.691, 1.308]</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.755645</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Estável</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Região: Sudeste</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0.0557</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1.0573</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[1.013, 1.103]</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.01041</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Crescente</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Região: Sul</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.0722</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1.0748</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>[0.989, 1.169]</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.09075800000000001</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Estável</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactoring modeling + shap
</commit_message>
<xml_diff>
--- a/resultados_estatisticos.xlsx
+++ b/resultados_estatisticos.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi2 e Cramer V" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mann-Whitney Salarial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spearman Nivel x Salario" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spearman Exp x Salario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tendencia Temporal" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1361,4 +1364,535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ρ (Senioridade × Salário)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>p-valor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Significativo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Magnitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9342</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2979</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.7178</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12321</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.7221</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ρ (Experiência × Salário)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>p-valor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Significativo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Magnitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10409</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6566</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3108</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.6296</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Geral</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>13517</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.6522</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Forte</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>β (log-odds/ano)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>IC 95% OR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p-valor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Significativo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>McFadden R²</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tendência</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Brasil — Geral</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17295</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0585</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.0603</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[1.025, 1.097]</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.000711</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Crescente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Região: Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1071</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1135</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.1202</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[0.971, 1.292]</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0.119501</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Estável</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Região: Nordeste</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1971</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0407</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.0415</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[0.940, 1.155]</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.439353</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Estável</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Região: Norte</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>256</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.0507</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[0.691, 1.308]</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.755645</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Estável</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Região: Sudeste</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10542</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0557</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.0573</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[1.013, 1.103]</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.01041</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Crescente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Região: Sul</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3044</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0722</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.0748</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[0.989, 1.169]</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.09075800000000001</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Estável</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
saving plots and refactoring details
</commit_message>
<xml_diff>
--- a/resultados_estatisticos.xlsx
+++ b/resultados_estatisticos.xlsx
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Usa IA gratuita (ChatGPT free)</t>
+          <t>Usa IA gratuita</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Usa Copilot / CodeWhisperer</t>
+          <t>Usa Copilot</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Usa IA gratuita (ChatGPT free)</t>
+          <t>Usa IA gratuita</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Usa Copilot / CodeWhisperer</t>
+          <t>Usa Copilot</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Usa IA gratuita (ChatGPT free)</t>
+          <t>Usa IA gratuita</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Usa Copilot / CodeWhisperer</t>
+          <t>Usa Copilot</t>
         </is>
       </c>
       <c r="C20" t="n">

</xml_diff>